<commit_message>
fix: remove repetitive 'Verify' prefix from all 300+ test case titles to ensure distinct, unique names in Excel
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Appium_Mobile_Automation_Report.xlsx
+++ b/Test Results/Excel/Appium_Mobile_Automation_Report.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Verify Android Fingerprint sensor prompt triggers on app launch</t>
+          <t>Fingerprint Sensor Prompt Trigger on Launch</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Verify Face Unlock authentication success unlocks mobile app dashboard</t>
+          <t>Face Unlock Dashboard Authentication</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Verify failed biometric authentication falls back to 4-digit PIN entry</t>
+          <t>Failed Biometric Fallback to 4-Digit PIN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Verify biometric hardware unavailable gracefully falls back to password</t>
+          <t>Hardware Unavailable Fallback to Password</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Verify invalid 4-digit PIN displays error toast notification</t>
+          <t>Invalid 4-Digit PIN Toast Error Alert</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Verify auto-lock mobile app after 60 seconds of device idle time</t>
+          <t>Auto-Lock Mobile App on 60s Idle Time</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Verify Android Keystore secure storage of user access tokens</t>
+          <t>Android Keystore Encrypted Access Token Storage</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Verify app lock screen hides sensitive posture preview thumbnail in recents app switcher</t>
+          <t>Recents Switcher Thumbnail Privacy Masking</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Verify biometric authentication setting toggle in security settings</t>
+          <t>Security Settings Biometric Toggle Switch</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Verify biometric re-authentication required before changing account password</t>
+          <t>Password Reset Biometric Re-Authentication</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Verify encrypted SQLite database initialization on first boot</t>
+          <t>Encrypted SQLite DB Initialization on First Boot</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Verify Certificate Pinning validation for HTTPS backend connections</t>
+          <t>Certificate Pinning HTTPS Connection Gate</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Verify root detection check displays security warning on rooted Android devices</t>
+          <t>Root Detection Security Warning Display</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Verify anti-tampering APK integrity signature check on app start</t>
+          <t>Anti-Tampering APK Integrity Signature Check</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Verify session timeout invalidates local biometric key cache</t>
+          <t>Session Timeout Local Key Cache Purge</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Verify PIN reset flow via registered mobile phone SMS verification code</t>
+          <t>SMS Verification Code PIN Reset Flow</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Verify Android screen capture restriction (FLAG_SECURE) on biometric prompt</t>
+          <t>FLAG_SECURE Screen Capture Restriction Check</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Verify app launch intent security check against malicious deep links</t>
+          <t>Deep Link App Launch Intent Security Filter</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Verify user logout purges OAuth refresh token from Android EncryptedSharedPreferences</t>
+          <t>OAuth Refresh Token Removal on Logout</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Verify account lockout after 5 consecutive failed PIN attempts</t>
+          <t>Account Lockout After 5 Failed Attempts</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Verify pattern unlock fallback configuration for legacy Android devices</t>
+          <t>Pattern Lock Fallback for Legacy Devices</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Verify biometric prompt cancellation leaves user on secure lock screen</t>
+          <t>Prompt Cancellation Lock Screen Security</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Verify multi-user Android device profile switching session separation</t>
+          <t>Multi-User Profile Switching Session Separation</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Verify biometrics registration update event invalidates cached session</t>
+          <t>Biometric Credential Update Event Handler</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Verify biometric prompt accessibility screen reader speech output</t>
+          <t>Screen Reader Speech Output for Biometrics</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Verify Android CAMERA runtime permission dialog request prompt</t>
+          <t>Runtime CAMERA Permission Request Dialog</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Verify front-facing selfie camera initializes default preview stream</t>
+          <t>Front Selfie Camera Default Preview Stream</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Verify rear-facing camera toggle switches active camera feed</t>
+          <t>Rear Camera Switch Button Interaction</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Verify Camera2 API high-frame-rate 60 FPS video capture initialization</t>
+          <t>Camera2 API 60 FPS High Frame Rate Engine</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Verify MediaPipe Android GPU acceleration module load speed</t>
+          <t>MediaPipe Android GPU Acceleration Initialization</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Verify 33 pose landmark coordinates rendered on Android SurfaceView</t>
+          <t>SurfaceView Render of 33 Pose Landmarks</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Verify camera autofocus adjustment in low-light indoor environments</t>
+          <t>Low-Light Indoor Camera Autofocus Adjustment</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Verify camera flash/flashlight toggle button on low-light detection</t>
+          <t>Flashlight Torch Toggle Button Activation</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Verify posture calibration wizard step 1 full body alignment box</t>
+          <t>Full Body Alignment Wizard Box Display</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Verify posture calibration wizard step 2 neck-to-ear angle check</t>
+          <t>Neck-to-Ear Lateral Angle Step Guidance</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Verify posture calibration wizard step 3 side-profile curvature check</t>
+          <t>Side-Profile Spine Curvature Wizard Step</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Verify live posture score HUD overlay updating at 30 FPS</t>
+          <t>HUD Overlay 30 FPS Live Posture Score Bar</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Verify camera resolution dynamic scaling based on Android battery saver mode</t>
+          <t>Battery Saver Mode Resolution Scaling</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Verify background camera pause when home button is pressed</t>
+          <t>Home Button Press Background Camera Pause</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Verify camera stream resumption when app is brought back to foreground</t>
+          <t>Foreground Resume Stream Re-Activation</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Verify portrait to landscape screen orientation camera stream reflow</t>
+          <t>Orientation Reflow Portrait to Landscape</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Verify multi-window split screen mode camera preview scaling</t>
+          <t>Multi-Window Split Screen Preview Layout</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Verify camera occlusion detection prompt when finger covers lens</t>
+          <t>Lens Occlusion Finger Detection Banner</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Verify face mesh landmark tracking synchronization with body pose</t>
+          <t>Face Mesh and Body Pose Sync Tracking</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Verify posture landmark confidence score filter (&gt;0.85 threshold)</t>
+          <t>Landmark Confidence Threshold Filter (&gt;0.85)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Verify camera hardware in use by another app graceful error handling</t>
+          <t>Hardware In-Use Conflict Exception Handling</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Verify image frame downsampling under high CPU thermal throttling</t>
+          <t>Thermal Throttling Frame Rate Downsampling</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Verify posture snapshot capture button saves screenshot to local gallery</t>
+          <t>Snapshot Capture Saved to Local Gallery</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Verify real-time slouch overlay skeleton color shift (Green -&gt; Red)</t>
+          <t>Slouch Skeleton Color Shift Green to Red</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Verify camera exposure compensation slider in settings</t>
+          <t>Exposure Compensation Setting Slider</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Verify wide-angle camera lens selection on multi-camera devices</t>
+          <t>Wide-Angle Lens Selection on Multi-Cam Devices</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Verify camera stream frame drop detection monitor (&lt;5% dropped frames)</t>
+          <t>Frame Drop Monitor (&lt;5% Dropped Frames)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Verify MediaPipe pose model switching between Light and Heavy models</t>
+          <t>Light vs Heavy MediaPipe Model Switch</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Verify camera preview aspect ratio fitting without visual distortion</t>
+          <t>Aspect Ratio Aspect Fitting Without Distortion</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Verify camera permission denied fallback screen with settings shortcut</t>
+          <t>Permission Denied Shortcut to Settings App</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Verify Android Vibrator service permission initialization</t>
+          <t>Vibrator System Service Initialization</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Verify short double-pulse haptic vibration on mild slouch detection</t>
+          <t>Short Double-Pulse Mild Slouch Warning</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Verify long continuous haptic vibration on severe posture slouch (&gt;10s)</t>
+          <t>Long Continuous Pulse Severe Slouch Alert</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Verify haptic feedback intensity slider control (Soft, Medium, Strong)</t>
+          <t>Vibration Intensity Control Slider (Soft/Strong)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Verify haptic feedback toggle switch in posture alert settings</t>
+          <t>Alert Settings Haptic Feedback Master Toggle</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Verify haptic pattern customization dropdown (Pulse, Heartbeat, Continuous)</t>
+          <t>Vibration Pattern Selector (Pulse/Heartbeat)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Verify Do Not Disturb (DND) system mode silences haptic vibrations</t>
+          <t>Do Not Disturb (DND) Vibration Suppression</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Verify haptic feedback test button triggers immediate sample vibration</t>
+          <t>Test Vibration Sample Trigger Button</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Verify haptic feedback suppression during phone call active state</t>
+          <t>Active Phone Call Haptic Mute Protection</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Verify smartwatch haptic notification sync via Android Wear OS bridge</t>
+          <t>Wear OS Smartwatch Haptic Notification Sync</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Verify haptic vibration delay setting (1s, 3s, 5s posture slouch delay)</t>
+          <t>Slouch Warning Delay Control (1s to 5s)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Verify haptic feedback battery impact optimization (&lt;1% battery per hour)</t>
+          <t>Battery Optimization Haptic Impact (&lt;1%/hr)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Verify vibration motor hardware missing fallback to audio alert</t>
+          <t>Hardware Missing Fallback to Audio Chime</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Verify haptic feedback trigger counter logging in daily posture stats</t>
+          <t>Daily Slouch Vibration Trigger Logging</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Verify haptic vibration mute during scheduled sleep hours</t>
+          <t>Scheduled Sleep Hours Haptic Suppression</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Verify haptic feedback on successful posture calibration completion</t>
+          <t>Calibration Completion Haptic Confirmation</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Verify subtle haptic tick feedback on slider movement in UI</t>
+          <t>UI Slider Touch Movement Haptic Tick</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Verify haptic feedback on tab bar item selection</t>
+          <t>Bottom Tab Bar Item Selection Haptic Click</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Verify haptic feedback on pull-to-refresh pull threshold reached</t>
+          <t>Pull-to-Refresh Threshold Haptic Pop</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Verify haptic feedback on posture goal milestone achieved modal</t>
+          <t>Milestone Unlocked Haptic Reward Feedback</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Verify Android POST_NOTIFICATIONS runtime permission prompt (Android 13+)</t>
+          <t>POST_NOTIFICATIONS Runtime Permission Prompt</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Verify Firebase Cloud Messaging (FCM) token registration on launch</t>
+          <t>FCM Device Registration Token Ingestion</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2938,7 +2938,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Verify foreground notification service channel setup for live tracking</t>
+          <t>Foreground Live Tracking Notification Channel</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Verify persistent status bar notification displaying real-time posture score</t>
+          <t>Status Bar Ongoing Live Posture Score Tile</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Verify tapping status bar notification opens posture live tracking screen</t>
+          <t>Status Bar Notification Tap Screen Launcher</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Verify posture slouch warning push notification payload reception</t>
+          <t>Posture Slouch Warning Push Payload Processing</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Verify hourly stretch reminder push notification display</t>
+          <t>Hourly Ergonomic Stretch Reminder Display</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Verify daily posture summary notification at 6:00 PM local time</t>
+          <t>Daily 6 PM Posture Digest Summary Notification</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3130,7 +3130,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Verify notification action button 'Pause Tracking' executes in background</t>
+          <t>Action Button 'Pause Tracking' Notification Execution</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Verify notification action button 'Mute 1 Hour' suppresses alerts</t>
+          <t>Action Button 'Mute 1 Hr' Alert Suppression</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Verify background posture tracking service survival under Android Doze mode</t>
+          <t>Doze Mode Background Service Survival</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Verify Android WorkManager periodic background posture sync task</t>
+          <t>WorkManager Periodic Background Sync Execution</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Verify notification LED light color customization (Green/Red)</t>
+          <t>Custom Notification LED Flash Color Configuration</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Verify notification sound custom ringtone playback</t>
+          <t>Ringtone Sound Selector Playback Preference</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Verify silent notification setting for background sync updates</t>
+          <t>Silent Notification Channel for Background Updates</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Verify clearing notifications from Android notification shade</t>
+          <t>Dismiss All Notifications Shade Action Handler</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Verify notification grouping for multiple posture slouch alerts</t>
+          <t>Slouch Warning Message Stacking and Grouping</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Verify notification priority level setting (HIGH for slouch warnings)</t>
+          <t>High Priority Channel Elevation for Slouch Alerts</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Verify background service restart on device boot (RECEIVE_BOOT_COMPLETED)</t>
+          <t>RECEIVE_BOOT_COMPLETED Auto-Start Service</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Verify background service termination when user stops posture tracking</t>
+          <t>Tracking Stop Action Background Service Lifecycle</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3514,7 +3514,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Verify FCM payload topic subscription for ergonomic wellness tips</t>
+          <t>FCM Wellness Tip Topic Subscription Sync</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Verify notification badge icon count increment on Android launcher</t>
+          <t>Launcher Icon Unread Notification Badge Count</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Verify push notification deep link navigation to specific session ID</t>
+          <t>Deep Link Route Navigation From Push Payload</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Verify notification delivery log in app diagnostic settings</t>
+          <t>App Diagnostic Notification Delivery Audit Log</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Verify background memory footprint under 50MB during passive tracking</t>
+          <t>Background Memory Retention Limit (&lt;50MB Footprint)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Verify swipe left gesture navigates to next posture analysis screen</t>
+          <t>Swipe Left Route Transition Gesture</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Verify swipe right gesture returns to previous posture screen</t>
+          <t>Swipe Right Back Navigation Transition</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Verify pull-to-refresh gesture on dashboard reloads posture metrics</t>
+          <t>Pull-to-Refresh Analytics Dashboard Reload</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Verify pinch-to-zoom gesture on posture angle timeline chart</t>
+          <t>Pinch-to-Zoom Posture Angle Chart Axis</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Verify double-tap gesture on video feed toggles full screen mode</t>
+          <t>Double-Tap Video Full Screen Mode Switch</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3834,7 +3834,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Verify long-press gesture on session history item opens action menu</t>
+          <t>Long-Press Session History Context Menu</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Verify swipe-to-delete gesture on session list row removes entry</t>
+          <t>Swipe-to-Delete Session List Item Action</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Verify Android edge-to-edge gesture navigation back swipe handling</t>
+          <t>Android Edge-to-Edge System Back Gesture</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Verify bottom sheet modal swipe down to dismiss gesture</t>
+          <t>Bottom Sheet Swipe Down Dismissal</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Verify drag scroll momentum on long session history list view</t>
+          <t>Kinetic Scroll Momentum on Long History Lists</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Verify touch target touch padding meets 48x48dp Android guidelines</t>
+          <t>Minimum 48x48dp Touch Target Size Compliance</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Verify ripple effect visual feedback on material button press</t>
+          <t>Material Ripple Tap Effect Animation</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -4058,7 +4058,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Verify double-tap prevention on action buttons during API requests</t>
+          <t>Button Double-Tap Prevention Safeguard</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Verify floating action button (FAB) hide on list scroll down</t>
+          <t>FAB Auto-Hide on List Scroll Down</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Verify FAB reveal on list scroll up</t>
+          <t>FAB Auto-Reveal on List Scroll Up</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Verify tab bar tap switches view without page reload flicker</t>
+          <t>Tab Bar Instant View Switch Without Flicker</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Verify tooltip popup display on long-press help icons</t>
+          <t>Help Icon Long-Press Tooltip Popover</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Verify slider thumb drag smooth value updating</t>
+          <t>Slider Thumb Drag Value Tracking</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -4250,7 +4250,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Verify multi-touch gesture rejection during active camera calibration</t>
+          <t>Multi-Touch Rejection During Active Calibration</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Verify gesture velocity threshold detection for quick swipe actions</t>
+          <t>Quick Swipe Velocity Threshold Recognition</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Verify back press hardware key handling closes open navigation drawer</t>
+          <t>Hardware Back Button Close Drawer Navigation</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Verify back press hardware key handling on home screen shows exit prompt</t>
+          <t>Hardware Back Button App Exit Modal Prompt</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Verify scroll position restoration on navigating back to dashboard</t>
+          <t>Scroll Position Persistence on Route Return</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -4410,7 +4410,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Verify carousel swipe indicator dot animation</t>
+          <t>Carousel Dots Indicator Slide Animation</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Verify expandable accordion list item expand/collapse tap gesture</t>
+          <t>Accordion Panel Expand and Collapse Gesture</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -4474,7 +4474,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Verify Android Bluetooth LE permission request dialog</t>
+          <t>Bluetooth LE Runtime Permission Request Prompt</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Verify scanning for nearby PostureFixPro BLE smart wearable devices</t>
+          <t>Scanning Nearby PostureFixPro Smart Wearables</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Verify BLE device connection handshake and pairing verification</t>
+          <t>BLE Handshake and Security Pairing Bond</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Verify real-time BLE accelerometer telemetry stream ingestion (50Hz)</t>
+          <t>50Hz BLE Accelerometer Raw Sensor Stream</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Verify real-time BLE gyroscope spinal tilt angle calculation</t>
+          <t>BLE Gyroscope Spinal Tilt Calculation Engine</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Verify BLE battery level indicator display in app status bar</t>
+          <t>Wearable Battery Percentage Status Bar Tile</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Verify BLE disconnection auto-reconnect retry loop</t>
+          <t>BLE Disconnection Auto-Reconnect Backoff</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -4698,7 +4698,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Verify wearable haptic motor trigger command sent over BLE</t>
+          <t>Haptic Alert Command Transmission Over BLE</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Verify BLE firmware update over-the-air (OTA) check</t>
+          <t>Over-The-Air (OTA) BLE Firmware Update Check</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Verify BLE connection loss alert banner display</t>
+          <t>BLE Connection Loss Status Banner Alert</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Verify wearable sensor calibration button zeroing spinal angles</t>
+          <t>Spinal Angle Sensor Zeroing Calibration Button</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Verify dual-sensor fusion (Camera + BLE Wearable) accuracy boost</t>
+          <t>Camera plus BLE Sensor Fusion Accuracy Boost</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Verify BLE data packet checksum integrity verification</t>
+          <t>Packet Checksum CRC Integrity Verification</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Verify unpairing BLE device removes stored MAC address</t>
+          <t>Wearable Device Unpairing and MAC Removal</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Verify BLE signal strength (RSSI) meter display</t>
+          <t>Signal Strength (RSSI) Signal Level Gauge</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -4954,7 +4954,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Verify BLE background sync service status</t>
+          <t>Background BLE Telemetry Sync Service Status</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Verify multiple BLE device pairing conflict resolution</t>
+          <t>Multiple Wearable Device Pairing Conflict Handling</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Verify BLE passkey authentication during initial bond</t>
+          <t>Passkey Input Pairing Authentication Screen</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -5050,7 +5050,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Verify BLE data logging to local encrypted SQLite table</t>
+          <t>Encrypted Local SQLite BLE Telemetry Logging</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Verify BLE device sleep mode wake-up interrupt event</t>
+          <t>Wearable Device Sleep Mode Interrupt Wakeup</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Verify SQLite database creation and schema migration v1 to v2</t>
+          <t>SQLite DB Schema Migration Version 1 to 2</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -5146,7 +5146,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Verify saving posture tracking sessions to local SQLite database when offline</t>
+          <t>Offline Session Saving to Local Encrypted Database</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Verify airplane mode detection triggers offline banner indicator</t>
+          <t>Airplane Mode Network Status Banner Toggle</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Verify automatic sync queue processing upon network reconnection</t>
+          <t>Network Reconnection Automatic Sync Dispatcher</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -5242,7 +5242,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Verify HTTP 500 backend error triggers retry backoff in sync queue</t>
+          <t>Backend HTTP 500 Retry Exponential Backoff</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -5274,7 +5274,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Verify local database record conflict resolution (Server-wins strategy)</t>
+          <t>Server-Wins Data Conflict Resolution Handler</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Verify offline posture score history chart rendering from SQLite data</t>
+          <t>Offline SQLite Historical Chart Renderer</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -5338,7 +5338,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Verify offline image asset caching in Android internal storage</t>
+          <t>Android Internal Cache Image Asset Storage</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Verify Room DB DAO insert query performance (&lt;10ms for 100 rows)</t>
+          <t>Room DB DAO Batch Insert (&lt;10ms Benchmark)</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -5402,7 +5402,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Verify database vacuum and optimization task on app startup</t>
+          <t>Database Vacuum Maintenance Task on Startup</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Verify max offline storage quota limit enforcement (50MB cap)</t>
+          <t>50MB Max Offline Storage Cap Enforcement</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Verify purging old offline sessions older than 90 days</t>
+          <t>Purge Offline Session Records Older Than 90 Days</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -5498,7 +5498,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Verify offline user settings modifications persist across app restarts</t>
+          <t>Offline Settings Changes Persistence Check</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -5530,7 +5530,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Verify sync status indicator icon (Synced, Syncing, Pending Offline)</t>
+          <t>Sync Status Indicator Icon (Synced/Pending)</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Verify manual 'Sync Now' button triggers immediate backend synchronization</t>
+          <t>Manual 'Sync Now' Action Button Ingestion</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Verify JSON payload serialization for batch offline session upload</t>
+          <t>JSON Batch Upload Payload Serialization</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Verify handling partial network failure mid-way through batch sync upload</t>
+          <t>Partial Upload Failure Recovery Queueing</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Verify database corruption recovery fallback database re-creation</t>
+          <t>Database Corruption Auto-Recovery Re-Creation</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Verify offline posture summary report PDF generation from local storage</t>
+          <t>Offline Local Report PDF File Generator</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -5722,7 +5722,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Verify offline analytics calculation accuracy matching backend server logic</t>
+          <t>Local Offline Analytics Logic Parity Check</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -5754,7 +5754,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Verify SQLite encrypted database password key retrieval from KeyStore</t>
+          <t>KeyStore Encryption Key Decryption Pass</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Verify background sync execution restriction on low battery (&lt;15%)</t>
+          <t>Low Battery (&lt;15%) Background Sync Suppression</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -5818,7 +5818,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Verify background sync execution restriction on metered mobile data</t>
+          <t>Metered Data Saver Connection Sync Deferral</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -5850,7 +5850,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Verify offline posture alert notification generation without server API</t>
+          <t>Standalone Offline Posture Alert Generator</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -5882,7 +5882,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Verify local DB export to external storage backup file (.db)</t>
+          <t>Local Database Backup Export to .DB File</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Verify MPAndroidChart daily posture score line chart rendering</t>
+          <t>MPAndroidChart Daily Posture Score Line Rendering</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Verify posture score marker popup on touching chart data node</t>
+          <t>Data Point Touch Marker Popup Display</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Verify weekly slouch distribution bar chart animation on screen enter</t>
+          <t>Weekly Slouch Bar Chart Entry Animation</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -6010,7 +6010,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Verify posture grade circular progress indicator (A, B, C, D, F)</t>
+          <t>Circular Progress Health Grade Badge (A-F)</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -6042,7 +6042,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Verify real-time posture index gauge updates smoothly during session</t>
+          <t>Real-Time Posture Index Gauge Smooth Needle Move</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -6074,7 +6074,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Verify top posture metrics cards (Avg Score, Slouch Time, Total Breaks)</t>
+          <t>Top Summary Metric Cards (Score/Slouch/Breaks)</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Verify quick action button 'Start Live Tracking' navigation</t>
+          <t>Quick Action 'Start Live Tracking' Button Tap</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -6138,7 +6138,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Verify quick action button 'Calibrate Camera' navigation</t>
+          <t>Quick Action 'Calibrate Camera' Button Tap</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Verify quick action button 'Upload Video' navigation</t>
+          <t>Quick Action 'Upload Video' Button Tap</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -6202,7 +6202,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Verify streak counter widget display with fire icon animation</t>
+          <t>Daily Posture Streak Counter Flame Animation</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Verify ergonomics tip card swipe to see next tip gesture</t>
+          <t>Ergonomics Tip Card Horizontal Swipe Gesture</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -6266,7 +6266,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Verify dashboard layout reflow on 5-inch vs 6.7-inch mobile screens</t>
+          <t>Layout Viewport Adaptation (5-inch vs 6.7-inch)</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Verify dashboard widget customization drag to reorder</t>
+          <t>Dashboard Drag-and-Drop Card Reordering</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Verify dark mode color scheme adaptation on charts and graphs</t>
+          <t>Dark Mode Native Chart Theme Adaptation</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Verify chart zoom reset button after pinch-to-zoom interaction</t>
+          <t>Reset Pinch Zoom Viewport Action Button</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -6394,7 +6394,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Verify dashboard empty state graphic when zero tracking data recorded</t>
+          <t>Zero Session Data Empty State Graphic Illustration</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -6426,7 +6426,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Verify dashboard swipe down pull-to-refresh animation feedback</t>
+          <t>Swipe Down Refresh Spinner Motion Feedback</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Verify posture health risk score warning alert card on dashboard</t>
+          <t>Health Risk Advisory Card for Low Posture Scores</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Verify total posture tracking time formatted string (e.g. 14h 30m)</t>
+          <t>Tracking Time Duration Text Formatter</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Verify quick date filter tabs (Day, Week, Month, Year)</t>
+          <t>Time Range Tabs Switcher (Day/Week/Month)</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -6554,7 +6554,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Verify active posture session status banner on top of dashboard</t>
+          <t>Active Session Tracking Banner Floating Bar</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -6586,7 +6586,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Verify dashboard network disconnection offline badge overlay</t>
+          <t>Network Offline Mode Warning Badge Bar</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -6618,7 +6618,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Verify posture achievement unlocked toast notification display</t>
+          <t>Achievement Unlocked Celebratory Toast Alert</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Verify posture goal target progress percentage bar</t>
+          <t>Daily Target Progress Ring Percentage Calculation</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Verify sharing posture dashboard summary screenshot to social apps</t>
+          <t>Social App Dashboard Image Share Dispatcher</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Verify dashboard memory retention check after 10 minutes of active use</t>
+          <t>Continuous 10-Minute Active View RAM Check</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -6746,7 +6746,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Verify high-contrast chart accessibility mode for color-blind users</t>
+          <t>High-Contrast Accessible Chart Mode Toggle</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Verify dashboard floating action button quick start camera tracking</t>
+          <t>Floating Action Button Camera Quick Trigger</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -6810,7 +6810,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Verify posture score calculation accuracy for multi-hour sessions</t>
+          <t>Multi-Hour Tracking Score Precision Engine</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Verify dashboard rendering performance under 60 FPS smooth scroll</t>
+          <t>Smooth 60 FPS Native Chart Scroll Benchmark</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -6874,7 +6874,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Verify Android READ_MEDIA_VIDEO permission request dialog</t>
+          <t>READ_MEDIA_VIDEO Permission Request Dialog</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Verify selecting posture video from Android system media gallery</t>
+          <t>System Media Picker Video File Selector</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -6938,7 +6938,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Verify Android FFmpeg video hardware acceleration transcoding</t>
+          <t>FFmpeg Hardware Accelerated Video Compression</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -6970,7 +6970,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Verify compressing 4K 60FPS video to 720p 30FPS before upload</t>
+          <t>4K 60FPS Video Transcoding Down to 720p 30FPS</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -7002,7 +7002,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Verify video file size reduction percentage metric output</t>
+          <t>File Size Savings Percentage Calculation</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Verify video trimming slider select start and end timestamps</t>
+          <t>Video Trimmer Start/End Timestamp Selector</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Verify video player play/pause state synchronization</t>
+          <t>Video Player Play and Pause Controls</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Verify video scrubbing seeker bar smooth frame preview</t>
+          <t>Seeker Bar Frame Thumbnail Hover Preview</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Verify uploading compressed video file to Cloudinary backend API</t>
+          <t>Cloudinary Backend Video Upload Dispatch</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -7162,7 +7162,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Verify upload progress bar percentage notification</t>
+          <t>Upload Percentage Notification Progress Bar</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Verify background video upload WorkManager task</t>
+          <t>Background WorkManager Video Upload Task</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -7226,7 +7226,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Verify uploading video over Wi-Fi only user setting toggle</t>
+          <t>Wi-Fi Only Video Upload Setting Restriction</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -7258,7 +7258,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Verify video upload error handling on broken connection</t>
+          <t>Network Drop Mid-Upload Connection Retry</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Verify video processing completion push notification alert</t>
+          <t>Video Analysis Processing Complete Push Alert</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -7322,7 +7322,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Verify posture angle landmark skeleton playback overlay on video</t>
+          <t>Landmark Skeleton Overlay Playback Sync</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -7354,7 +7354,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Verify video analysis report summary card rendering</t>
+          <t>Post-Upload Video AI Report Card Display</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -7386,7 +7386,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Verify deleting uploaded posture video from local device cache</t>
+          <t>Delete Uploaded Video File From Local Storage</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -7418,7 +7418,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Verify corrupted video file detection before upload start</t>
+          <t>Corrupted Video Bitstream Early Rejection</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -7450,7 +7450,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Verify video upload cancellation cleans up temporary swap files</t>
+          <t>Upload Cancel Temp Swap File Cleanup</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -7482,7 +7482,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Verify maximum video duration restriction (max 10 minutes)</t>
+          <t>Maximum Video Length Limit (10 Minutes) Gate</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Verify minimum video duration restriction (min 5 seconds)</t>
+          <t>Minimum Video Length Limit (5 Seconds) Gate</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Verify audio track stripping from video during compression for privacy</t>
+          <t>Audio Channel Stripping for Privacy Protection</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Verify video thumbnail extraction from 1st second keyframe</t>
+          <t>First Frame Keyframe Thumbnail Extraction</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -7610,7 +7610,7 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Verify video player orientation flip on device rotation</t>
+          <t>Device Rotation Video Aspect Ratio Flip</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -7642,7 +7642,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Verify video analysis result comparison side-by-side view</t>
+          <t>Side-by-Side Video Posture Comparison View</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Verify gracefully handling permission denied permanently (Never Ask Again)</t>
+          <t>Permanent Permission Denied Settings Reroute</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -7706,7 +7706,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Verify app permission settings shortcut button launches Android App Settings</t>
+          <t>Android Settings App Shortcut Button Launch</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -7738,7 +7738,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Verify Android 14 granular media permissions (Photos &amp; Videos)</t>
+          <t>Android 14 Granular Media Files Permission</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Verify Android 12 exact alarm permission for scheduled posture alerts</t>
+          <t>Android 12 Exact Alarm Permission Handling</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -7802,7 +7802,7 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Verify background location permission rejection does not crash camera</t>
+          <t>Location Permission Denial Fallback Gate</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Verify Android battery optimization exemption prompt for tracking service</t>
+          <t>Battery Optimization Exemption Request Flow</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -7866,7 +7866,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Verify Android storage permission (WRITE_EXTERNAL_STORAGE) legacy support</t>
+          <t>Legacy External Storage Permission Check</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -7898,7 +7898,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Verify Android microphone permission request for voice command posture controls</t>
+          <t>Voice Control Microphone Permission Dialog</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -7930,7 +7930,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Verify runtime permission status re-check on every app resume</t>
+          <t>App Resume Permission State Verification</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -7962,7 +7962,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Verify camera permission revocation while app in background handles state</t>
+          <t>Background Camera Revocation Safety Catch</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Verify Android multi-window mode UI responsive reflow</t>
+          <t>Android Split Screen Multi-Tasking Reflow</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -8026,7 +8026,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Verify Android foldable device hinge folding state layout update</t>
+          <t>Foldable Device Screen Hinge Fold Event</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Verify Android tablet 10-inch screen dual-pane master-detail layout</t>
+          <t>10-inch Tablet Master-Detail Dual Pane View</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Verify Android TV / ChromeOS non-touch screen keyboard navigation</t>
+          <t>Android TV D-Pad Focus Navigation Support</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -8122,7 +8122,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Verify low RAM device (&lt;2GB RAM) low-memory warning handler</t>
+          <t>Low Memory Device (&lt;2GB RAM) Warning Handler</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Verify Android thermal status listener throttling intensive AI processing</t>
+          <t>Thermal Status Listener AI Engine Throttle</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Verify dark theme system setting change auto-updates mobile app theme</t>
+          <t>System Dark Theme Auto-Switch Adaptation</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -8218,7 +8218,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Verify system font scale size change scales mobile app typography cleanly</t>
+          <t>System Font Scaling Dynamic Text Resize</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -8250,7 +8250,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Verify locale language change (English -&gt; Spanish) auto-reloads app strings</t>
+          <t>Locale Switch String Localization Reload</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -8282,7 +8282,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Verify right-to-left (RTL) layout mirroring for Arabic locale</t>
+          <t>RTL Arabic Mirroring UI Orientation Check</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -8314,7 +8314,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Verify mobile app startup time cold boot under 1.5 seconds</t>
+          <t>Cold Boot App Launch Time (&lt;1.5s Benchmark)</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -8346,7 +8346,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Verify mobile app startup time warm boot under 0.5 seconds</t>
+          <t>Warm Boot App Resume Time (&lt;0.5s Benchmark)</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -8378,7 +8378,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Verify CPU usage under 25% during active camera posture tracking</t>
+          <t>CPU Utilization During Active Camera Tracking (&lt;25%)</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -8410,7 +8410,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Verify RAM usage under 150MB during active camera posture tracking</t>
+          <t>RAM Footprint During Active Tracking (&lt;150MB)</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -8442,7 +8442,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Verify zero memory leaks after 50 activity screen transitions</t>
+          <t>Zero Memory Leak Check After 50 Transitions</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Verify battery consumption under 3% per 30 minutes of tracking</t>
+          <t>Battery Drain Rate (&lt;3% per 30 Mins)</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -8506,7 +8506,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Verify GPU memory release when closing camera tracking screen</t>
+          <t>GPU Context Release on Camera View Destroy</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -8538,7 +8538,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Verify background service CPU consumption under 1% when idle</t>
+          <t>Background Service Passive Idle CPU (&lt;1%)</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -8570,7 +8570,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Verify network data consumption under 100 KB per posture session</t>
+          <t>Network Data Traffic Consumption (&lt;100KB/session)</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -8602,7 +8602,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Verify Android ANR (Application Not Responding) zero occurrences during heavy AI processing</t>
+          <t>Zero ANR (Application Not Responding) Pass</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -8634,7 +8634,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Verify Android strict mode zero disk read/write violations on main thread</t>
+          <t>StrictMode Main Thread Disk I/O Check</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -8666,7 +8666,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Verify bitmap image caching and recycling prevents OutOfMemoryError</t>
+          <t>Bitmap Garbage Recycling OutOfMemory Safety</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -8698,7 +8698,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Verify database connection pool closure on app destroy</t>
+          <t>SQLite Connection Pool Closure on Teardown</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -8730,7 +8730,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Verify background thread executor pool termination on app exit</t>
+          <t>ThreadPool Executor Shutdown on Exit</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Verify frame rendering rate stays locked at 60 FPS during list scrolling</t>
+          <t>List Scroll Smooth 60 FPS Frame Lock</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -8794,7 +8794,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Verify low battery mode (&lt;15%) automatically reduces MediaPipe FPS to 15 FPS</t>
+          <t>Low Battery (&lt;15%) Auto FPS Reduction to 15 FPS</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -8826,7 +8826,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Verify app APK bundle size under 35MB (optimized with ProGuard/R8)</t>
+          <t>Optimized APK Bundle Size (&lt;35MB Package)</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -8858,7 +8858,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Verify ProGuard obfuscation strips unused code and debug logging</t>
+          <t>ProGuard R8 Dead Code Stripping Check</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -8890,7 +8890,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Verify native C++ OpenCV library memory management stability</t>
+          <t>Native C++ OpenCV Memory Allocation Safety</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Verify garbage collection pauses under 10ms during continuous tracking</t>
+          <t>Garbage Collection Pause Duration (&lt;10ms)</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Verify automatic HTTP request retry backoff on 3G to 4G handover</t>
+          <t>Network Handover 3G to 4G Request Retry</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Verify handling total packet loss during active live telemetry post</t>
+          <t>Total Packet Loss Resilience Handling</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Verify SSL handshake timeout error toast notification display</t>
+          <t>SSL Handshake Timeout Dialog Prompt</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -9050,7 +9050,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Verify socket connection reset error graceful recovery without crashing</t>
+          <t>Socket Connection Reset Graceful Catch</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -9082,7 +9082,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Verify captive portal Wi-Fi network detection display warning</t>
+          <t>Captive Portal Wi-Fi Detection Banner</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Verify DNS resolution failure fallback to cached IP address</t>
+          <t>DNS Resolution Failure Fallback IP Connect</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -9146,7 +9146,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Verify slow 2G network throttle simulated API timeout handling</t>
+          <t>Slow 2G Speed Connection Timeout Alert</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -9178,7 +9178,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Verify airplane mode toggle mid-upload pauses and queues upload</t>
+          <t>Mid-Upload Airplane Toggle Pause Queue</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -9210,7 +9210,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Verify VPN network adapter interface state change detection</t>
+          <t>VPN Network Adapter Switch Re-Handshake</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -9242,7 +9242,7 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Verify IPv6 to IPv4 dual-stack network socket failover</t>
+          <t>IPv6 Dual-Stack Network Socket Failover</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -9269,12 +9269,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Verify Wear OS companion app pairing discovery over Bluetooth LE</t>
+          <t>Smartwatch BLE Discovery and Pairing Flow</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -9301,12 +9301,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Verify posture slouch haptic alert sync to Wear OS smartwatch wrist motor</t>
+          <t>Slouch Warning Wrist Vibration Sync</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -9333,12 +9333,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Verify Wear OS watch face complication displays real-time posture score</t>
+          <t>Watch Face Complication Score Indicator</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -9365,12 +9365,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Verify Wear OS heart rate telemetry stream correlation with posture stress</t>
+          <t>Heart Rate Sensor Stress Correlation Sync</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -9397,12 +9397,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Verify Wear OS quick action tile 'Pause Tracking' command reception</t>
+          <t>Quick Tile 'Pause Tracking' Remote Trigger</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -9429,12 +9429,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Verify Wear OS standalone mode posture tracking without active phone link</t>
+          <t>Standalone Smartwatch Posture Mode Without Phone</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -9461,12 +9461,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Verify Wear OS low-power ambient display mode UI optimization</t>
+          <t>Ambient Low-Power Watch Display Mode</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -9493,12 +9493,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Verify Wear OS notification dismiss sync to handheld smartphone app</t>
+          <t>Smartwatch Notification Dismiss Handheld Sync</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -9525,12 +9525,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Verify Wear OS battery drain under 2% per hour during posture tracking</t>
+          <t>Watch Battery Drain Rate (&lt;2%/hr) Test</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -9557,12 +9557,12 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Wear OS Integration</t>
+          <t>Smartwatch Wear OS</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Verify Wear OS sensor calibration tap gesture prompt</t>
+          <t>Wrist Sensor Zero Alignment Tap Prompt</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -9594,7 +9594,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Verify Spanish locale string translations on dashboard UI</t>
+          <t>Spanish Language Dashboard String Set</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -9626,7 +9626,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Verify French locale string translations on posture calibration UI</t>
+          <t>French Language Calibration Screen Text</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -9658,7 +9658,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Verify German locale string translations on settings screen</t>
+          <t>German Language Settings Screen Layout</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -9690,7 +9690,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Verify Japanese locale character rendering without text clipping</t>
+          <t>Japanese Kana Text Rendering Clip Check</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -9722,7 +9722,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Verify Chinese Simplified string translation formatting</t>
+          <t>Chinese Simplified Character Set Encoding</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -9754,7 +9754,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Verify Hindi locale string translations on alert settings</t>
+          <t>Hindi Language Alert Settings Strings</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -9786,7 +9786,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Verify Portuguese locale number formatting (comma decimal separator)</t>
+          <t>Portuguese Decimal Formatter (Comma Sep)</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -9818,7 +9818,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Verify Arabic RTL layout mirroring on bottom navigation bar</t>
+          <t>RTL Arabic Navigation Layout Mirroring</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -9850,7 +9850,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Verify date-time locale formatting (MM/DD/YYYY vs DD/MM/YYYY)</t>
+          <t>Localized Date-Time Format Parsing</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Verify currency symbol formatting on premium subscription page</t>
+          <t>Localized Currency Symbol Billing Page</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -9909,12 +9909,12 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Verify app process killed by Android OS Low Memory Killer state restoration</t>
+          <t>Low Memory Killer Process State Restore</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -9941,12 +9941,12 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Verify opening app via custom scheme deep link (posturefix://session/123)</t>
+          <t>Custom Scheme Deep Link (posturefix://)</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -9973,12 +9973,12 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Verify Universal Link URL handling from web browser to mobile app</t>
+          <t>Universal Web Link Navigation Handler</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -10005,12 +10005,12 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Verify app update prompt display when mandatory forced update is published</t>
+          <t>Mandatory Forced App Update Gate Screen</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
@@ -10037,12 +10037,12 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Verify in-app Google Play Store review prompt trigger after 10 sessions</t>
+          <t>In-App Play Store Review Trigger Prompt</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
@@ -10069,12 +10069,12 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Verify app shortcut long-press menu on Android launcher (Start Tracking)</t>
+          <t>Launcher Quick Action Long-Press Menu</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
@@ -10101,12 +10101,12 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Verify Android splash screen transition animation smoothness</t>
+          <t>Android Native Splash Screen Motion</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
@@ -10133,12 +10133,12 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Verify background task scheduling via Android AlarmManager</t>
+          <t>AlarmManager Scheduled Background Task</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
@@ -10165,12 +10165,12 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Verify app exit back press confirmation double-tap dialog</t>
+          <t>Double-Tap Back Exit Confirmation Dialog</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
@@ -10197,12 +10197,12 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>App Life-Cycle &amp; Deep Links</t>
+          <t>App Lifecycle &amp; Intent</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Verify cold launch intent parameter parsing for notification payload</t>
+          <t>Notification Payload Launch Parameter Intent</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">

</xml_diff>